<commit_message>
Export ESG : retirer les noms définis orphelins du gabarit (vraie cause de corruption)
Le gabarit Admaius contenait ~26 definedName pointant vers un classeur EXTERNE
absent ('[1]Underlying scores'!...). À l'ouverture, Excel tentait de résoudre
ces liens externes, échouait, et réclamait une réparation — malgré le retrait
des commentaires. Gabarit reconstruit sans noms définis ni liens externes ;
XML validé, sharedStrings cohérent.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/app/(app)/esg/_lib/esg-template.xlsx
+++ b/src/app/(app)/esg/_lib/esg-template.xlsx
@@ -8,37 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly data" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-  </externalReferences>
-  <definedNames>
-    <definedName name="CountryList">'[1]Underlying scores'!$P$4:$P$58</definedName>
-    <definedName name="Exclusions">'[1]Underlying scores'!$W$4:$W$6</definedName>
-    <definedName name="Externalities1">'[1]Underlying scores'!$D$9:$D$12</definedName>
-    <definedName name="Externalities2">'[1]Underlying scores'!$G$9:$G$11</definedName>
-    <definedName name="Externalities3">'[1]Underlying scores'!$J$9:$J$11</definedName>
-    <definedName name="Externalities4">'[1]Underlying scores'!$M$9:$M$11</definedName>
-    <definedName name="Externalities5">'[1]Underlying scores'!#REF!</definedName>
-    <definedName name="Gender1">'[1]Underlying scores'!$D$15:$D$18</definedName>
-    <definedName name="Gender2">'[1]Underlying scores'!$G$15:$G$18</definedName>
-    <definedName name="Gender3">'[1]Underlying scores'!$J$15:$J$18</definedName>
-    <definedName name="Gender4">'[1]Underlying scores'!$M$15:$M$18</definedName>
-    <definedName name="List0">'[1]Underlying scores'!$D$4:$D$6</definedName>
-    <definedName name="List1">'[1]Underlying scores'!$G$4:$G$5</definedName>
-    <definedName name="List2">'[1]Underlying scores'!$J$4:$J$6</definedName>
-    <definedName name="List4">'[1]Underlying scores'!#REF!</definedName>
-    <definedName name="ListBoxOutput">#REF!</definedName>
-    <definedName name="ListBoxOutput2">#REF!</definedName>
-    <definedName name="ListBoxOutput3">#REF!</definedName>
-    <definedName name="look">#REF!</definedName>
-    <definedName name="OutputHistorical1">#REF!</definedName>
-    <definedName name="OutputHistorical2">#REF!</definedName>
-    <definedName name="OutputHistorical3">#REF!</definedName>
-    <definedName name="ThematicSectors">'[1]Underlying scores'!$T$4:$T$9</definedName>
-    <definedName name="Work2">'[1]Underlying scores'!$G$21:$G$23</definedName>
-    <definedName name="Work3">'[1]Underlying scores'!$J$21:$J$23</definedName>
-    <definedName name="Work4">'[1]Underlying scores'!$M$21:$M$23</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -557,37 +527,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <sheetNames>
-      <sheetName val="1. Impact assessment"/>
-      <sheetName val="2. ESG assessment"/>
-      <sheetName val="NOT ALWAYS USED"/>
-      <sheetName val="REFERENCE tabs&gt;&gt;&gt;"/>
-      <sheetName val="Underlying scores"/>
-      <sheetName val="UNDP - HDI data"/>
-      <sheetName val="ND-GAIN - climate index"/>
-      <sheetName val="ND-GAIN - climate index ADJ GDP"/>
-      <sheetName val="Admaius priorities"/>
-      <sheetName val="Underlying_scores"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>